<commit_message>
Root-domain cleanup: Kuwait fashion stores
</commit_message>
<xml_diff>
--- a/markets/fashion/Kuwait_Fashion_Stores.xlsx
+++ b/markets/fashion/Kuwait_Fashion_Stores.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fashion Stores" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage &amp; Method" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Removed - platform subdomain" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26660,7 +26661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -27003,7 +27004,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -27013,6 +27013,94 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>Removed 2 rows from Fashion Stores (now 116); each is listed in the Excluded sheet with source "Deliverable cleanup (fashion-stores package)". Website values normalised to clean storefront URLs (2 changed). Counts above (total, type, gender, platform, size tier, verification status) reflect the cleaned list; any by-source/by-channel/signal-origin/QA breakdowns are as at the original run (pre-cleanup). Note: the Boutiqaat judgment call described above was resolved by removing it (beauty-led hybrid marketplace).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Root-domain cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rows before</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Kept as-is</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Replaced with root domain</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Removed (no own domain / duplicate of root)</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Rows after</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>116</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Store Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Old URL</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Reason</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recount page counts: retry failed child sitemaps, resolve zero-count market segments
</commit_message>
<xml_diff>
--- a/markets/fashion/Kuwait_Fashion_Stores.xlsx
+++ b/markets/fashion/Kuwait_Fashion_Stores.xlsx
@@ -1687,11 +1687,11 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0</v>
+        <v>22704</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>sitemap (KW pages only)</t>
+          <t>sitemap (partial: 27 of 28 sitemap files read)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2205,11 +2205,11 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>0</v>
+        <v>16424</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>sitemap (KW pages only)</t>
+          <t>sitemap (partial: 85 of 86 sitemap files read)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -3046,11 +3046,11 @@
         </is>
       </c>
       <c r="C41" s="3" t="n">
-        <v>0</v>
+        <v>512564</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>sitemap (KW pages only)</t>
+          <t>sitemap (whole site, no market segment)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3952,7 +3952,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>sitemap</t>
+          <t>sitemap (partial: 5 of 9 sitemap files read)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -28130,7 +28130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -28580,7 +28580,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45">
@@ -28596,89 +28596,89 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>sitemap (partial: some child sitemaps unreadable)</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>sitemap (whole site, no market segment)</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>Not available</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B48" t="n">
         <v>29</v>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>Size distribution (pages per site)</t>
         </is>
       </c>
-      <c r="B48" s="1" t="inlineStr">
+      <c r="B50" s="1" t="inlineStr">
         <is>
           <t>Rows</t>
         </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>1-50</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>51-200</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>201-1,000</t>
+          <t>1-50</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1,001-5,000</t>
+          <t>51-200</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>5,001-20,000</t>
+          <t>201-1,000</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>5</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>20,001-100,000</t>
+          <t>1,001-5,000</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>10</v>
+        <v>28</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>&gt;100,000</t>
+          <t>5,001-20,000</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -28688,23 +28688,33 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>0 (market segment empty)</t>
+          <t>20,001-100,000</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="58" ht="95" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>Method rules: sitemap counted in full (all child sitemaps followed); image and video sitemaps skipped; URLs deduplicated; Arabic and English URLs counted separately; when a sitemap is country-segmented only the listed market's pages are counted; fallbacks, used when no sitemap yields URLs, are the shop-page total, the platform product count (Shopify/WooCommerce) and the web archive (own host only); blocked or unreachable sites are marked Not available and left blank.</t>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>&gt;100,000</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" ht="150" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Method rules: sitemap counted in full (all child sitemaps followed); image and video sitemaps skipped; URLs deduplicated; Arabic and English URLs counted separately; when a sitemap is country-segmented only the listed market's pages are counted; fallbacks, used when no sitemap yields URLs, are the shop-page total, the platform product count (Shopify/WooCommerce) and the web archive (own host only); blocked or unreachable sites are marked Not available and left blank. Child sitemaps that failed are retried up to 4 times (5s/15s/45s/120s); if some still fail the row reads 'sitemap (partial: N of M sitemap files read)' and the count is a lower bound. If the sitemap has country segments but none for the listed market, the whole site is counted when a default storefront exists ('sitemap (whole site, no market segment)', which includes other-country URLs), otherwise the row is Not available.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A58:C58"/>
+    <mergeCell ref="A59:C59"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge rerun page counts into page count columns and coverage block
</commit_message>
<xml_diff>
--- a/markets/fashion/Kuwait_Fashion_Stores.xlsx
+++ b/markets/fashion/Kuwait_Fashion_Stores.xlsx
@@ -4654,10 +4654,12 @@
           <t>https://gcc.luluhypermarket.com/en-kw/</t>
         </is>
       </c>
-      <c r="C66" s="3" t="n"/>
+      <c r="C66" s="3" t="n">
+        <v>6839</v>
+      </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Not available (unreachable (ConnectionError: HTTPConnectionPool(host='www.gcc.luluhypermarket.com', port=80): Max retries exc))</t>
+          <t>archive</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -28558,7 +28560,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43">
@@ -28590,7 +28592,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46">
@@ -28620,7 +28622,7 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="50">
@@ -28682,7 +28684,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="56">

</xml_diff>

<commit_message>
KW fashion: add 8 StoreLeads gap-fill stores, excluded rows, coverage block, page counts
</commit_message>
<xml_diff>
--- a/markets/fashion/Kuwait_Fashion_Stores.xlsx
+++ b/markets/fashion/Kuwait_Fashion_Stores.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M117"/>
+  <dimension ref="A1:M125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -7993,6 +7993,526 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Leia</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>https://activeleia.com/</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>233</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Small / local brand</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>https://activeleia.com/products/zipper-jacket-set</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Aidan Global</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>https://aidanglobal.com/</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>796</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>WooCommerce</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Small / local brand</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>https://aidanglobal.com/product/premium-racefit-cycling-jersey-corex/</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Aurellia Official</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>https://aurelliaofficial.com/</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>10</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Small / local brand</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>https://aurelliaofficial.com/products/caramel-sweater-dark-chocolate-leather-skirt</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Black Line</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>https://blacklinewear.com/</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>73</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Unisex</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>OpenCart</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Small / local brand</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>https://blacklinewear.com/</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Doe</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>https://doekw.com/</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>archive</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Women, Men</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Not detected</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Small / local brand</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>https://doekw.com/en/products/4/men-clothing</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Hamem Design</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>https://hamemdesign.com/</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>142</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Small / local brand</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>https://hamemdesign.com/products/عباة-ميلا-بني-أو-أسود</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Maisonr</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>https://maisonrkw.com/</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>35</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Shopify</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Small / local brand</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>https://maisonrkw.com/</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ShopFlain</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>https://shopflain.com/</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>17039</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>archive</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Fashion-only</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>nopCommerce</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Verified – StoreLeads gap check</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>https://shopflain.com/pants-3</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>homepage/nav clothing keywords (StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8004,7 +8524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D914"/>
+  <dimension ref="A1:D967"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -28118,6 +28638,1172 @@
       <c r="D914" t="inlineStr">
         <is>
           <t>Deliverable cleanup (fashion-stores package)</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>3DPRINT</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>https://www.3dprintkw.com/</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>53Sports &amp; Fitness</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>https://53sports.com/</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>albairaqkw</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>https://www.albairaqkw.com/</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>albayrouni Pharmacy</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>https://albayrouni-pharmacy.com.kw/</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>All Drops Store</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>https://www.alldrops.store/</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D919" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>Alsultan Pharmacy</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>https://www.alsultanpharmacy.com/</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>Althenayan Honey</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>http://althenayanhoney.com/</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>Anesthesia Contact Lenses</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>http://anesthesialenses.com/</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>ArabiaScents</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>https://arabiascents.com/</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>أريج الكويت للعطور</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>https://areejkw.com/</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>أطيب الدولية</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>https://atiabintl.com/</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>Beautica Cosmetics</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>https://www.beautica-cosmetics.com/</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>Bella Contact Lenses</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>https://bellacontactlenses.com/</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>BLOCK7.STORE</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>https://block7.store/</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>BoardGames Q8</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>https://boardgamesq8.com/</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D929" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>By Talal</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>https://bytalal.com/</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>Carmen Professional</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>https://carmenprofessional.com/</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>eBaqala.com</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>https://ebaqala.com/</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>FAWAAH</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>https://fawaah.com/</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>Findik Nuts</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>https://findiknuts.com/</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>fnbyfn</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>https://fnbyfn.com/</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>فريسيا</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>https://freesia-beauty.com/</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>GAMESQ8.com</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>https://gamesq8.com/</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>Ginza Market Kuwait</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>https://www.ginzamartkw.com/</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>Henzadem</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>https://henzadem.com/</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D939" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>H&amp;S Store</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>https://hsstore.com/</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>آي سيلكت</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>https://iselectkw.com/</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>Kent Web Store Kuwait</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>https://kentwebstore.com/</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>Kuwait Diet</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>https://kuwait-diet.com/</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>Loroyal Color contact</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>https://loroyallenses.com/</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>مزهاف</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>https://mzhaf.com/</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>Noor Foods KW</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>https://noororganicfood.com/</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>Noor Organic Q8</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>https://noororganicq8.com/</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>PERFUME KUWAIT</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>https://otorkuwit.com/</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>Perfumes600</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>https://perfumes600.com/</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D949" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>Pharmazone</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>https://pharmazone.com/</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>Puchi Box</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>https://puchi-kw.com/</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>REGAL HONEY</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>https://regal-honey.com/</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>Sedra</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>https://sedrahoney.com/</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>Sedra Perfumes</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>https://www.sedraperfumes.com/</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>Sincerely Jules</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>https://sincerelyjuleskw.com/</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>Smart Collection</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>https://smartcollectionkw.com/</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>Smart Hydro</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>https://smarthydro.net/</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>ستايلاتي</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>https://stylati.com/</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>Telefonati</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>https://www.telefonati.com/</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>The Honey Garden</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>https://thehoneygarden.com/</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>The Shop Wings</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>https://theshopwings.com/</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>Trust Pharmacy</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>https://thetrustpharmacy.com/</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>Tula Aloud</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>https://tula-aloud.com/</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>tum.tum.tam</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>https://www.tumtumtam.com/</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>Twenty Five</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>https://twentyfive.com.kw/</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>ugreenkuwait</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>https://ugreenkuwait.com/</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>ZwarahHome</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>https://zwarahhome.com/</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>no clothing signal (added by StoreLeads gap fill)</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill</t>
         </is>
       </c>
     </row>
@@ -28132,7 +29818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -28171,7 +29857,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>124</t>
         </is>
       </c>
     </row>
@@ -28546,89 +30232,100 @@
         <v>116</v>
       </c>
     </row>
+    <row r="38"/>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>Page count</t>
+          <t>StoreLeads gap fill</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Rows counted (of 116)</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>88</v>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>StoreLeads gap fill of the Kuwait directory (see directory workbook, sheet 'Research Coverage')</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Gap stores added to the directory</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t>Counted by method</t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>Rows</t>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Gap stores added to the fashion list</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>sitemap</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>74</v>
+          <t>Gap stores not fashion (listed in Excluded)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>archive</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>sitemap (partial: some child sitemaps unreadable)</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>3</v>
-      </c>
-    </row>
+          <t>Fashion rules</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Adult clothing (women, men, unisex) as a fashion-only store or a clothing section; abaya/thobe/modest wear, lingerie and sportswear count; kids-only and shoes/bags/accessories-only do not. Classified from homepage nav/meta and product pages (EN+AR keywords), reviewed manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>sitemap (whole site, no market segment)</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>1</v>
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>Page count</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Not available</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>28</v>
-      </c>
-    </row>
+          <t>Rows counted (of 124)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
-          <t>Size distribution (pages per site)</t>
+          <t>Counted by method</t>
         </is>
       </c>
       <c r="B50" s="1" t="inlineStr">
@@ -28640,75 +30337,162 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1-50</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>9</v>
+          <t>sitemap</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>51-200</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>9</v>
+          <t>archive</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>201-1,000</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>17</v>
+          <t>sitemap (partial: some child sitemaps unreadable)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1,001-5,000</t>
-        </is>
-      </c>
-      <c r="B54" t="n">
-        <v>28</v>
+          <t>sitemap (whole site, no market segment)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>Not available</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="56"/>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>Size distribution (pages per site)</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1-50</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>51-200</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>201-1,000</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1,001-5,000</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>5,001-20,000</t>
         </is>
       </c>
-      <c r="B55" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>20,001-100,000</t>
         </is>
       </c>
-      <c r="B56" t="n">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>&gt;100,000</t>
         </is>
       </c>
-      <c r="B57" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="59" ht="150" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="150" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Method rules: sitemap counted in full (all child sitemaps followed); image and video sitemaps skipped; URLs deduplicated; Arabic and English URLs counted separately; when a sitemap is country-segmented only the listed market's pages are counted; fallbacks, used when no sitemap yields URLs, are the shop-page total, the platform product count (Shopify/WooCommerce) and the web archive (own host only); blocked or unreachable sites are marked Not available and left blank. Child sitemaps that failed are retried up to 4 times (5s/15s/45s/120s); if some still fail the row reads 'sitemap (partial: N of M sitemap files read)' and the count is a lower bound. If the sitemap has country segments but none for the listed market, the whole site is counted when a default storefront exists ('sitemap (whole site, no market segment)', which includes other-country URLs), otherwise the row is Not available.</t>
         </is>
@@ -28716,7 +30500,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A66:C66"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>